<commit_message>
feat: land SkillCast, InSave equip/magicbook UI, and visual model scale (v0.82.75)
PushMap auto-casts Skill_03/01/02, InSave shell exposes equipment warehouse and magic-book reorder, and Mode2 soldiers bake VisualModelScale with AllIn1 styles.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CursorGame_Git\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Mode2\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12280"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="74">
   <si>
     <t>魔法书ID</t>
   </si>
@@ -181,10 +181,7 @@
     <t>装备后，Mode2 制造的枯骨战士/战士主属性增加躯体该维之和的 15%（可叠），至彻底死亡</t>
   </si>
   <si>
-    <t>Style_WarriorGlow</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>Style_ScaleModel</t>
   </si>
   <si>
     <t>MagicBook_SoldierSkillLevel</t>
@@ -221,12 +218,6 @@
   </si>
   <si>
     <t>装备后，Mode2 制造职业为 Class_BaseWarrior 的士兵时，变为 Class_Warrior</t>
-  </si>
-  <si>
-    <t>Style_AdvanceOutline</t>
-  </si>
-  <si>
-    <t>30</t>
   </si>
   <si>
     <t>MagicBook_ArcherAdvance</t>
@@ -737,148 +728,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1235,12 +1226,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="9" max="9" width="29.6363636363636" customWidth="1"/>
-    <col min="10" max="10" width="23.6363636363636" customWidth="1"/>
-    <col min="11" max="11" width="16.6363636363636" customWidth="1"/>
-    <col min="12" max="12" width="21.5454545454545" customWidth="1"/>
+    <col min="8" max="8" width="16.75" customWidth="1"/>
+    <col min="9" max="9" width="29.6333333333333" customWidth="1"/>
+    <col min="10" max="10" width="23.6333333333333" customWidth="1"/>
+    <col min="11" max="11" width="16.6333333333333" customWidth="1"/>
+    <col min="12" max="12" width="21.5416666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1385,8 +1377,6 @@
       <c r="I4" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
@@ -1419,16 +1409,16 @@
       <c r="J5" t="s">
         <v>49</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>37</v>
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1.5</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
         <v>38</v>
@@ -1440,25 +1430,25 @@
         <v>39</v>
       </c>
       <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
         <v>52</v>
-      </c>
-      <c r="F6" t="s">
-        <v>53</v>
       </c>
       <c r="G6" t="s">
         <v>41</v>
       </c>
       <c r="H6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" t="s">
         <v>54</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>55</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>37</v>
@@ -1466,7 +1456,7 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
@@ -1478,33 +1468,26 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="G7" t="s">
         <v>41</v>
       </c>
       <c r="H7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" t="s">
         <v>61</v>
       </c>
-      <c r="I7" t="s">
-        <v>62</v>
-      </c>
-      <c r="J7" t="s">
-        <v>63</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
@@ -1516,33 +1499,26 @@
         <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G8" t="s">
         <v>41</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
-      </c>
-      <c r="J8" t="s">
-        <v>63</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>37</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
@@ -1554,33 +1530,26 @@
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
         <v>41</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" t="s">
-        <v>63</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>37</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
         <v>37</v>
@@ -1592,29 +1561,22 @@
         <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s">
         <v>41</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I10" t="s">
-        <v>76</v>
-      </c>
-      <c r="J10" t="s">
-        <v>63</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>37</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>